<commit_message>
docs: Document ignored Sparkline formatting
</commit_message>
<xml_diff>
--- a/example/comparison.xlsx
+++ b/example/comparison.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,13 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>=1+2 -&gt; =2+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>=1+1 -&gt; =2+1</t>
         </is>
       </c>
     </row>
@@ -494,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>.\example\a.xlsx</t>
+          <t>example\a.xlsx</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -507,7 +514,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>.\example\b.xlsx</t>
+          <t>example\b.xlsx</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>

</xml_diff>